<commit_message>
electronica: Gebiete mit Zuständigen (Stefan BW, Dietmar Bayern)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBhay9ftM7ciQ2MUqqBU5G
</commit_message>
<xml_diff>
--- a/aussendienst/electronica_2026_Aussendienst.xlsx
+++ b/aussendienst/electronica_2026_Aussendienst.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zielfirmen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baden-Württemberg" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bayern" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baden-Württemberg (Stefan)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bayern (Dietmar)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rest DE - NL" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eher nicht (kein Bereich)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nicht ansprechen" sheetId="6" state="visible" r:id="rId6"/>
@@ -18,10 +18,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Zielfirmen'!$A$4:$K$205</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Zielfirmen'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Baden-Württemberg'!$A$4:$K$58</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Baden-Württemberg'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bayern'!$A$4:$K$51</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Bayern'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Baden-Württemberg (Stefan)'!$A$4:$K$58</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Baden-Württemberg (Stefan)'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bayern (Dietmar)'!$A$4:$K$51</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Bayern (Dietmar)'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rest DE - NL'!$A$4:$K$104</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Rest DE - NL'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Eher nicht (kein Bereich)'!$A$4:$I$295</definedName>
@@ -10550,7 +10550,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zielfirmen electronica 2026 – Baden-Württemberg</t>
+          <t>Zielfirmen electronica 2026 – Baden-Württemberg (Stefan)</t>
         </is>
       </c>
     </row>
@@ -10636,7 +10636,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -10685,7 +10685,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -10832,7 +10832,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -10930,7 +10930,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -10979,7 +10979,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -11028,7 +11028,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -11077,7 +11077,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -11126,7 +11126,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -11175,7 +11175,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -11224,7 +11224,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -11420,7 +11420,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -11469,7 +11469,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -11567,7 +11567,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -11616,7 +11616,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -11665,7 +11665,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -11714,7 +11714,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -11861,7 +11861,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -11959,7 +11959,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -12008,7 +12008,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -12106,7 +12106,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -12204,7 +12204,7 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -12253,7 +12253,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -12302,7 +12302,7 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -12400,7 +12400,7 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -12449,7 +12449,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -12498,7 +12498,7 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -12547,7 +12547,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -12596,7 +12596,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -12645,7 +12645,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
@@ -12792,7 +12792,7 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -12841,7 +12841,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -12890,7 +12890,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
@@ -13086,7 +13086,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -13184,7 +13184,7 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
@@ -13296,7 +13296,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zielfirmen electronica 2026 – Bayern</t>
+          <t>Zielfirmen electronica 2026 – Bayern (Dietmar)</t>
         </is>
       </c>
     </row>
@@ -13382,7 +13382,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -13431,7 +13431,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -13480,7 +13480,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -13578,7 +13578,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -13627,7 +13627,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -13823,7 +13823,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -13872,7 +13872,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -13921,7 +13921,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -13970,7 +13970,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -14068,7 +14068,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -14117,7 +14117,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -14166,7 +14166,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -14215,7 +14215,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -14264,7 +14264,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -14362,7 +14362,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -14411,7 +14411,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -14509,7 +14509,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -14558,7 +14558,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -14656,7 +14656,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -14803,7 +14803,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -14852,7 +14852,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -14950,7 +14950,7 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -14999,7 +14999,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -15048,7 +15048,7 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -15097,7 +15097,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -15146,7 +15146,7 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -15195,7 +15195,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -15244,7 +15244,7 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -15293,7 +15293,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -15391,7 +15391,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -15440,7 +15440,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -15489,7 +15489,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
@@ -15538,7 +15538,7 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -15636,7 +15636,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -34538,7 +34538,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -34585,7 +34585,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -34960,7 +34960,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -35140,7 +35140,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -35320,7 +35320,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -35562,7 +35562,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -35656,7 +35656,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -35703,7 +35703,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -35750,7 +35750,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -35797,7 +35797,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -35938,7 +35938,7 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -36032,7 +36032,7 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -36157,7 +36157,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -36290,7 +36290,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -36337,7 +36337,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -36384,7 +36384,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -36509,7 +36509,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -36728,7 +36728,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -36775,7 +36775,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -37002,7 +37002,7 @@
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -37049,7 +37049,7 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -37096,7 +37096,7 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -37143,7 +37143,7 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -37190,7 +37190,7 @@
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -37237,7 +37237,7 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -37284,7 +37284,7 @@
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -37331,7 +37331,7 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -37378,7 +37378,7 @@
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -38011,7 +38011,7 @@
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -38292,7 +38292,7 @@
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -38378,7 +38378,7 @@
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -38511,7 +38511,7 @@
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
@@ -38558,7 +38558,7 @@
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -38890,7 +38890,7 @@
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -39078,7 +39078,7 @@
       </c>
       <c r="D109" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -39211,7 +39211,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E112" s="11" t="inlineStr">
@@ -39258,7 +39258,7 @@
       </c>
       <c r="D113" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -39305,7 +39305,7 @@
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E114" s="11" t="inlineStr">
@@ -39352,7 +39352,7 @@
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -39704,7 +39704,7 @@
       </c>
       <c r="D123" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -39790,7 +39790,7 @@
       </c>
       <c r="D125" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
@@ -40083,7 +40083,7 @@
       <c r="C132" s="10" t="inlineStr"/>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E132" s="11" t="inlineStr">
@@ -40130,7 +40130,7 @@
       </c>
       <c r="D133" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -40255,7 +40255,7 @@
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E136" s="11" t="inlineStr">
@@ -40341,7 +40341,7 @@
       </c>
       <c r="D138" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E138" s="11" t="inlineStr">
@@ -40685,7 +40685,7 @@
       </c>
       <c r="D146" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E146" s="11" t="inlineStr">
@@ -40849,7 +40849,7 @@
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E150" s="11" t="inlineStr">
@@ -40935,7 +40935,7 @@
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E152" s="11" t="inlineStr">
@@ -41146,7 +41146,7 @@
       </c>
       <c r="D157" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E157" s="8" t="inlineStr">
@@ -41318,7 +41318,7 @@
       </c>
       <c r="D161" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E161" s="8" t="inlineStr">
@@ -41412,7 +41412,7 @@
       </c>
       <c r="D163" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E163" s="8" t="inlineStr">
@@ -41553,7 +41553,7 @@
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E166" s="11" t="inlineStr">
@@ -41811,7 +41811,7 @@
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E172" s="11" t="inlineStr">
@@ -41999,7 +41999,7 @@
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E176" s="11" t="inlineStr">
@@ -42124,7 +42124,7 @@
       </c>
       <c r="D179" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E179" s="8" t="inlineStr">
@@ -42210,7 +42210,7 @@
       </c>
       <c r="D181" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E181" s="8" t="inlineStr">
@@ -42335,7 +42335,7 @@
       </c>
       <c r="D184" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E184" s="11" t="inlineStr">
@@ -42382,7 +42382,7 @@
       </c>
       <c r="D185" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E185" s="8" t="inlineStr">
@@ -42507,7 +42507,7 @@
       </c>
       <c r="D188" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E188" s="11" t="inlineStr">
@@ -42593,7 +42593,7 @@
       </c>
       <c r="D190" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E190" s="11" t="inlineStr">
@@ -42687,7 +42687,7 @@
       </c>
       <c r="D192" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E192" s="11" t="inlineStr">
@@ -42734,7 +42734,7 @@
       </c>
       <c r="D193" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E193" s="8" t="inlineStr">
@@ -42867,7 +42867,7 @@
       </c>
       <c r="D196" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E196" s="11" t="inlineStr">
@@ -43008,7 +43008,7 @@
       </c>
       <c r="D199" s="8" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E199" s="8" t="inlineStr">
@@ -43133,7 +43133,7 @@
       </c>
       <c r="D202" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E202" s="11" t="inlineStr">
@@ -43219,7 +43219,7 @@
       </c>
       <c r="D204" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E204" s="11" t="inlineStr">
@@ -43305,7 +43305,7 @@
       </c>
       <c r="D206" s="11" t="inlineStr">
         <is>
-          <t>Bayern</t>
+          <t>Bayern (Dietmar)</t>
         </is>
       </c>
       <c r="E206" s="11" t="inlineStr">
@@ -43438,7 +43438,7 @@
       </c>
       <c r="D209" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E209" s="8" t="inlineStr">
@@ -43524,7 +43524,7 @@
       </c>
       <c r="D211" s="8" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E211" s="8" t="inlineStr">
@@ -43571,7 +43571,7 @@
       </c>
       <c r="D212" s="11" t="inlineStr">
         <is>
-          <t>Baden-Württemberg</t>
+          <t>Baden-Württemberg (Stefan)</t>
         </is>
       </c>
       <c r="E212" s="11" t="inlineStr">
@@ -43888,7 +43888,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Tom/Tina. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
+          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Tom/Tina. Zuständig: Stefan = Baden-Württemberg, Dietmar = Bayern. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
electronica: Manuel für Rest DE/NL
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBhay9ftM7ciQ2MUqqBU5G
</commit_message>
<xml_diff>
--- a/aussendienst/electronica_2026_Aussendienst.xlsx
+++ b/aussendienst/electronica_2026_Aussendienst.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zielfirmen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baden-Württemberg (Stefan)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bayern (Dietmar)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rest DE - NL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rest DE - NL (Manuel)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eher nicht (kein Bereich)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nicht ansprechen" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="7" state="visible" r:id="rId7"/>
@@ -22,8 +22,8 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Baden-Württemberg (Stefan)'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bayern (Dietmar)'!$A$4:$K$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Bayern (Dietmar)'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rest DE - NL'!$A$4:$K$104</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Rest DE - NL'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rest DE - NL (Manuel)'!$A$4:$K$104</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Rest DE - NL (Manuel)'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Eher nicht (kein Bereich)'!$A$4:$I$295</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Eher nicht (kein Bereich)'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Nicht ansprechen'!$A$4:$I$215</definedName>
@@ -15699,7 +15699,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zielfirmen electronica 2026 – Rest DE / NL</t>
+          <t>Zielfirmen electronica 2026 – Rest DE / NL (Manuel)</t>
         </is>
       </c>
     </row>
@@ -15785,7 +15785,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -15883,7 +15883,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -15932,7 +15932,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -15981,7 +15981,7 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -16079,7 +16079,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -16177,7 +16177,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -16226,7 +16226,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -16275,7 +16275,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -16324,7 +16324,7 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -16373,7 +16373,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -16422,7 +16422,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -16471,7 +16471,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -16520,7 +16520,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -16569,7 +16569,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -16618,7 +16618,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -16667,7 +16667,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -16716,7 +16716,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
@@ -16863,7 +16863,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
@@ -16961,7 +16961,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -17010,7 +17010,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -17108,7 +17108,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
@@ -17157,7 +17157,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -17206,7 +17206,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -17255,7 +17255,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
@@ -17353,7 +17353,7 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -17402,7 +17402,7 @@
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -17500,7 +17500,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -17549,7 +17549,7 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -17598,7 +17598,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -17647,7 +17647,7 @@
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -17696,7 +17696,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -17794,7 +17794,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
@@ -17843,7 +17843,7 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -17892,7 +17892,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
@@ -17941,7 +17941,7 @@
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -18039,7 +18039,7 @@
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -18088,7 +18088,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -18137,7 +18137,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -18186,7 +18186,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -18284,7 +18284,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -18333,7 +18333,7 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -18382,7 +18382,7 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
@@ -18431,7 +18431,7 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -18480,7 +18480,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -18529,7 +18529,7 @@
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -18578,7 +18578,7 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -18627,7 +18627,7 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -18676,7 +18676,7 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
@@ -18725,7 +18725,7 @@
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -18774,7 +18774,7 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -18823,7 +18823,7 @@
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -18872,7 +18872,7 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
@@ -18921,7 +18921,7 @@
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -18970,7 +18970,7 @@
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -19019,7 +19019,7 @@
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -19117,7 +19117,7 @@
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -19166,7 +19166,7 @@
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -19215,7 +19215,7 @@
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -19264,7 +19264,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
@@ -19313,7 +19313,7 @@
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -19362,7 +19362,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
@@ -19411,7 +19411,7 @@
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -19460,7 +19460,7 @@
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
@@ -19509,7 +19509,7 @@
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -19558,7 +19558,7 @@
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
@@ -19607,7 +19607,7 @@
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -19656,7 +19656,7 @@
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
@@ -19705,7 +19705,7 @@
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -19754,7 +19754,7 @@
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -19852,7 +19852,7 @@
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
@@ -19901,7 +19901,7 @@
       </c>
       <c r="D89" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -19950,7 +19950,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
@@ -19999,7 +19999,7 @@
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -20048,7 +20048,7 @@
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -20097,7 +20097,7 @@
       </c>
       <c r="D93" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -20146,7 +20146,7 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -20195,7 +20195,7 @@
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -20244,7 +20244,7 @@
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
@@ -20293,7 +20293,7 @@
       </c>
       <c r="D97" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -20342,7 +20342,7 @@
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
@@ -20391,7 +20391,7 @@
       </c>
       <c r="D99" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -20440,7 +20440,7 @@
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
@@ -20489,7 +20489,7 @@
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -20538,7 +20538,7 @@
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
@@ -20587,7 +20587,7 @@
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -20636,7 +20636,7 @@
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
@@ -34632,7 +34632,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -34679,7 +34679,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -35093,7 +35093,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -35273,7 +35273,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -35609,7 +35609,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -35844,7 +35844,7 @@
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -36243,7 +36243,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
@@ -36595,7 +36595,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -36681,7 +36681,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
@@ -36822,7 +36822,7 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -36908,7 +36908,7 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -36955,7 +36955,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
@@ -37589,7 +37589,7 @@
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -37714,7 +37714,7 @@
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -37878,7 +37878,7 @@
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -37964,7 +37964,7 @@
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -38425,7 +38425,7 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
@@ -38757,7 +38757,7 @@
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
@@ -38804,7 +38804,7 @@
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -38937,7 +38937,7 @@
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
@@ -38984,7 +38984,7 @@
       </c>
       <c r="D107" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -39031,7 +39031,7 @@
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
@@ -39164,7 +39164,7 @@
       </c>
       <c r="D111" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -39399,7 +39399,7 @@
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
@@ -39446,7 +39446,7 @@
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -39610,7 +39610,7 @@
       </c>
       <c r="D121" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
@@ -39657,7 +39657,7 @@
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
@@ -39837,7 +39837,7 @@
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E126" s="11" t="inlineStr">
@@ -39923,7 +39923,7 @@
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E128" s="11" t="inlineStr">
@@ -40427,7 +40427,7 @@
       </c>
       <c r="D140" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E140" s="11" t="inlineStr">
@@ -40474,7 +40474,7 @@
       </c>
       <c r="D141" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -41099,7 +41099,7 @@
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E156" s="11" t="inlineStr">
@@ -41271,7 +41271,7 @@
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E160" s="11" t="inlineStr">
@@ -41365,7 +41365,7 @@
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E162" s="11" t="inlineStr">
@@ -41459,7 +41459,7 @@
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E164" s="11" t="inlineStr">
@@ -41506,7 +41506,7 @@
       </c>
       <c r="D165" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E165" s="8" t="inlineStr">
@@ -41600,7 +41600,7 @@
       </c>
       <c r="D167" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E167" s="8" t="inlineStr">
@@ -41725,7 +41725,7 @@
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E170" s="11" t="inlineStr">
@@ -41858,7 +41858,7 @@
       </c>
       <c r="D173" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E173" s="8" t="inlineStr">
@@ -41905,7 +41905,7 @@
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E174" s="11" t="inlineStr">
@@ -41952,7 +41952,7 @@
       </c>
       <c r="D175" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E175" s="8" t="inlineStr">
@@ -42640,7 +42640,7 @@
       </c>
       <c r="D191" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E191" s="8" t="inlineStr">
@@ -42820,7 +42820,7 @@
       </c>
       <c r="D195" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E195" s="8" t="inlineStr">
@@ -42914,7 +42914,7 @@
       </c>
       <c r="D197" s="8" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E197" s="8" t="inlineStr">
@@ -42961,7 +42961,7 @@
       </c>
       <c r="D198" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E198" s="11" t="inlineStr">
@@ -43391,7 +43391,7 @@
       </c>
       <c r="D208" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E208" s="11" t="inlineStr">
@@ -43657,7 +43657,7 @@
       </c>
       <c r="D214" s="11" t="inlineStr">
         <is>
-          <t>Rest DE / NL</t>
+          <t>Rest DE / NL (Manuel)</t>
         </is>
       </c>
       <c r="E214" s="11" t="inlineStr">
@@ -43888,7 +43888,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Tom/Tina. Zuständig: Stefan = Baden-Württemberg, Dietmar = Bayern. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
+          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Tom/Tina. Zuständig: Stefan = Baden-Württemberg, Dietmar = Bayern, Manuel = Rest DE / NL. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
electronica: Außendienst-Excel final (interne Begriffe bereinigt)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBhay9ftM7ciQ2MUqqBU5G
</commit_message>
<xml_diff>
--- a/aussendienst/electronica_2026_Aussendienst.xlsx
+++ b/aussendienst/electronica_2026_Aussendienst.xlsx
@@ -4452,7 +4452,7 @@
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K74" s="11" t="inlineStr"/>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K85" s="8" t="inlineStr"/>
@@ -7746,7 +7746,7 @@
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K135" s="8" t="inlineStr"/>
@@ -11683,12 +11683,12 @@
       </c>
       <c r="I208" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Zeile "alfatec GmbH &amp; Co. KG" (Zeile 72) bzw. "alfatec" (Zeile 71) dieselbe Gruppe/Anschrift wie ai-energy (Meckenloher Str. 11)? Und welche Rolle hat Hitachi/Eigene Harze (Bestandskontakt)? Wo: CRM-Datensatz …</t>
+          <t>Intern klären: Ist die CRM-Zeile "alfatec GmbH &amp; Co. KG" (Zeile 72) bzw. "alfatec" (Zeile 71) dieselbe Gruppe/Anschrift wie ai-energy (Meckenloher Str. 11)? Und welche Rolle hat Hitachi/Eigene Harze (Bestandskontakt)? Wo: CRM-Datensatz …</t>
         </is>
       </c>
       <c r="J208" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K208" s="11" t="inlineStr"/>
@@ -11899,12 +11899,12 @@
       </c>
       <c r="I212" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist AUMOVIO Germany GmbH Rechtsnachfolgerin/umfirmierte Einheit der CRM-Zeile "Continental Automotive Technologies GmbH" bzw. steht "Continental" (Zeile 442) für dieselbe Gruppe?</t>
+          <t>Intern klären: Ist AUMOVIO Germany GmbH Rechtsnachfolgerin/umfirmierte Einheit der CRM-Zeile "Continental Automotive Technologies GmbH" bzw. steht "Continental" (Zeile 442) für dieselbe Gruppe?</t>
         </is>
       </c>
       <c r="J212" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K212" s="11" t="inlineStr"/>
@@ -11953,7 +11953,7 @@
       </c>
       <c r="I213" s="8" t="inlineStr">
         <is>
-          <t>Jey: Gehört BDT Pfronten heute noch zur AdCapital AG, und ist der CRM-Bestandskontakt (Erich Jaeger, EW HOF, FRAKO oder TALLER) für Pfronten ohne Bedeutung (eigene Gesellschaft, anderer Ansprechpartner)?</t>
+          <t>Intern klären: Gehört BDT Pfronten heute noch zur AdCapital AG, und ist der CRM-Bestandskontakt (Erich Jaeger, EW HOF, FRAKO oder TALLER) für Pfronten ohne Bedeutung (eigene Gesellschaft, anderer Ansprechpartner)?</t>
         </is>
       </c>
       <c r="J213" s="8" t="inlineStr">
@@ -12169,7 +12169,7 @@
       </c>
       <c r="I217" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Zeile "electronic concept GmbH" (bekannte_firmen, Z. 637) die Gaggenauer Gesellschaft, die jetzt zur elbe Gruppe gehört?</t>
+          <t>Intern klären: Ist die CRM-Zeile "electronic concept GmbH" (bekannte_firmen, Z. 637) die Gaggenauer Gesellschaft, die jetzt zur elbe Gruppe gehört?</t>
         </is>
       </c>
       <c r="J217" s="8" t="inlineStr">
@@ -12277,12 +12277,12 @@
       </c>
       <c r="I219" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist CRM-Zeile 737 "ETS" (und 2036 "S.E. System Electronic") dieselbe Einheit wie ET System electronic GmbH, Altlußheim?</t>
+          <t>Intern klären: Ist CRM-Zeile 737 "ETS" (und 2036 "S.E. System Electronic") dieselbe Einheit wie ET System electronic GmbH, Altlußheim?</t>
         </is>
       </c>
       <c r="J219" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K219" s="8" t="inlineStr"/>
@@ -12385,7 +12385,7 @@
       </c>
       <c r="I221" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist die Bürkert GmbH &amp; Co. KG im CRM (Zeile 366) Bestandskontakt der Bürkert-Gruppe, und gilt die Fäth GmbH als Schwester/Beteiligung (Rot E5 nur bei derselben Einheit; sonst Neukontakt nach Jeys Entscheidung)?</t>
+          <t>Intern klären: Ist die Bürkert GmbH &amp; Co. KG im CRM (Zeile 366) Bestandskontakt der Bürkert-Gruppe, und gilt die Fäth GmbH als Schwester/Beteiligung (Rot E5 nur bei derselben Einheit; sonst Neukontakt nach interner Entscheidung)?</t>
         </is>
       </c>
       <c r="J221" s="8" t="inlineStr">
@@ -12547,12 +12547,12 @@
       </c>
       <c r="I224" s="11" t="inlineStr">
         <is>
-          <t>(a) Jey bestätigt, dass HEIDEN electronics GmbH (Amtsgericht Augsburg B15917) als Zielgesellschaft aufgenommen wird (HEIDEN power GmbH = Vertrieb). (b) Fertigung durch die electronics-GmbH in Pürgen mit eigener Quelle belegen …</t>
+          <t>(a) intern bestätigen, dass HEIDEN electronics GmbH (Amtsgericht Augsburg B15917) als Zielgesellschaft aufgenommen wird (HEIDEN power GmbH = Vertrieb). (b) Fertigung durch die electronics-GmbH in Pürgen mit eigener Quelle belegen …</t>
         </is>
       </c>
       <c r="J224" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K224" s="11" t="inlineStr"/>
@@ -12606,7 +12606,7 @@
       </c>
       <c r="J225" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K225" s="8" t="inlineStr"/>
@@ -12763,12 +12763,12 @@
       </c>
       <c r="I228" s="11" t="inlineStr">
         <is>
-          <t>Jey: Steht im CRM die Bosch-Einheit "Bosch Security Systems/Building Technologies" (Grasbrunn/Straubing) oder nur andere Bosch-Gesellschaften (Robert Bosch GmbH, Rexroth, Power Tools)?</t>
+          <t>Intern klären: Steht im CRM die Bosch-Einheit "Bosch Security Systems/Building Technologies" (Grasbrunn/Straubing) oder nur andere Bosch-Gesellschaften (Robert Bosch GmbH, Rexroth, Power Tools)?</t>
         </is>
       </c>
       <c r="J228" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K228" s="11" t="inlineStr"/>
@@ -13038,7 +13038,7 @@
       </c>
       <c r="J233" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K233" s="8" t="inlineStr"/>
@@ -13087,12 +13087,12 @@
       </c>
       <c r="I234" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist MAIR Elektronik GmbH im CRM als Teil von RAWE Electronic GmbH (Zeile 1948) oder Demmel AG (Zeile 501) bereits betreut?</t>
+          <t>Intern klären: Ist MAIR Elektronik GmbH im CRM als Teil von RAWE Electronic GmbH (Zeile 1948) oder Demmel AG (Zeile 501) bereits betreut?</t>
         </is>
       </c>
       <c r="J234" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K234" s="11" t="inlineStr"/>
@@ -13249,7 +13249,7 @@
       </c>
       <c r="I237" s="8" t="inlineStr">
         <is>
-          <t>An Jey: Ist die CRM-Zeile "J. Schneider Elektrotechnik" (Z. 1208, Offenburg?) die Offenburger Schwester der Huber SE? Wenn ja: Konzernbezug zu einem Bestandskunden, Vorgehen mit Jey/Vertrieb abstimmen (kein Neukunde im Sinne E5 …</t>
+          <t>Intern klären: Ist die CRM-Zeile "J. Schneider Elektrotechnik" (Z. 1208, Offenburg?) die Offenburger Schwester der Huber SE? Wenn ja: Konzernbezug zu einem Bestandskunden, Vorgehen mit dem Vertrieb abstimmen (kein Neukunde im Sinne E5 …</t>
         </is>
       </c>
       <c r="J237" s="8" t="inlineStr">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="I245" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Einheit "VON ARDENNE GmbH" (Dresden) Gesellschafterin/Muttergesellschaft der scia Systems GmbH, und gilt der Bestandskontakt auch für scia?</t>
+          <t>Intern klären: Ist die CRM-Einheit "VON ARDENNE GmbH" (Dresden) Gesellschafterin/Muttergesellschaft der scia Systems GmbH, und gilt der Bestandskontakt auch für scia?</t>
         </is>
       </c>
       <c r="J245" s="8" t="inlineStr">
@@ -13789,12 +13789,12 @@
       </c>
       <c r="I247" s="8" t="inlineStr">
         <is>
-          <t>Jey: Welche Gesellschaft steht hinter CRM-Zeilen "Sumitomo"/"SUMITOMO" (2273/2274)? Gehört sie zur Sumitomo-Electric-Gruppe?</t>
+          <t>Intern klären: Welche Gesellschaft steht hinter CRM-Zeilen "Sumitomo"/"SUMITOMO" (2273/2274)? Gehört sie zur Sumitomo-Electric-Gruppe?</t>
         </is>
       </c>
       <c r="J247" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K247" s="8" t="inlineStr"/>
@@ -17297,7 +17297,7 @@
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Zeile "electronic concept GmbH" (bekannte_firmen, Z. 637) die Gaggenauer Gesellschaft, die jetzt zur elbe Gruppe gehört?</t>
+          <t>Intern klären: Ist die CRM-Zeile "electronic concept GmbH" (bekannte_firmen, Z. 637) die Gaggenauer Gesellschaft, die jetzt zur elbe Gruppe gehört?</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
@@ -17405,12 +17405,12 @@
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist CRM-Zeile 737 "ETS" (und 2036 "S.E. System Electronic") dieselbe Einheit wie ET System electronic GmbH, Altlußheim?</t>
+          <t>Intern klären: Ist CRM-Zeile 737 "ETS" (und 2036 "S.E. System Electronic") dieselbe Einheit wie ET System electronic GmbH, Altlußheim?</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K61" s="8" t="inlineStr"/>
@@ -17518,7 +17518,7 @@
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K63" s="8" t="inlineStr"/>
@@ -17675,7 +17675,7 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>An Jey: Ist die CRM-Zeile "J. Schneider Elektrotechnik" (Z. 1208, Offenburg?) die Offenburger Schwester der Huber SE? Wenn ja: Konzernbezug zu einem Bestandskunden, Vorgehen mit Jey/Vertrieb abstimmen (kein Neukunde im Sinne E5 …</t>
+          <t>Intern klären: Ist die CRM-Zeile "J. Schneider Elektrotechnik" (Z. 1208, Offenburg?) die Offenburger Schwester der Huber SE? Wenn ja: Konzernbezug zu einem Bestandskunden, Vorgehen mit dem Vertrieb abstimmen (kein Neukunde im Sinne E5 …</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
@@ -18974,7 +18974,7 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr"/>
@@ -19784,7 +19784,7 @@
       </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr"/>
@@ -20643,12 +20643,12 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Zeile "alfatec GmbH &amp; Co. KG" (Zeile 72) bzw. "alfatec" (Zeile 71) dieselbe Gruppe/Anschrift wie ai-energy (Meckenloher Str. 11)? Und welche Rolle hat Hitachi/Eigene Harze (Bestandskontakt)? Wo: CRM-Datensatz …</t>
+          <t>Intern klären: Ist die CRM-Zeile "alfatec GmbH &amp; Co. KG" (Zeile 72) bzw. "alfatec" (Zeile 71) dieselbe Gruppe/Anschrift wie ai-energy (Meckenloher Str. 11)? Und welche Rolle hat Hitachi/Eigene Harze (Bestandskontakt)? Wo: CRM-Datensatz …</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K54" s="11" t="inlineStr"/>
@@ -20805,12 +20805,12 @@
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist AUMOVIO Germany GmbH Rechtsnachfolgerin/umfirmierte Einheit der CRM-Zeile "Continental Automotive Technologies GmbH" bzw. steht "Continental" (Zeile 442) für dieselbe Gruppe?</t>
+          <t>Intern klären: Ist AUMOVIO Germany GmbH Rechtsnachfolgerin/umfirmierte Einheit der CRM-Zeile "Continental Automotive Technologies GmbH" bzw. steht "Continental" (Zeile 442) für dieselbe Gruppe?</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K57" s="8" t="inlineStr"/>
@@ -20859,7 +20859,7 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Jey: Gehört BDT Pfronten heute noch zur AdCapital AG, und ist der CRM-Bestandskontakt (Erich Jaeger, EW HOF, FRAKO oder TALLER) für Pfronten ohne Bedeutung (eigene Gesellschaft, anderer Ansprechpartner)?</t>
+          <t>Intern klären: Gehört BDT Pfronten heute noch zur AdCapital AG, und ist der CRM-Bestandskontakt (Erich Jaeger, EW HOF, FRAKO oder TALLER) für Pfronten ohne Bedeutung (eigene Gesellschaft, anderer Ansprechpartner)?</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
@@ -20967,12 +20967,12 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>(a) Jey bestätigt, dass HEIDEN electronics GmbH (Amtsgericht Augsburg B15917) als Zielgesellschaft aufgenommen wird (HEIDEN power GmbH = Vertrieb). (b) Fertigung durch die electronics-GmbH in Pürgen mit eigener Quelle belegen …</t>
+          <t>(a) intern bestätigen, dass HEIDEN electronics GmbH (Amtsgericht Augsburg B15917) als Zielgesellschaft aufgenommen wird (HEIDEN power GmbH = Vertrieb). (b) Fertigung durch die electronics-GmbH in Pürgen mit eigener Quelle belegen …</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr"/>
@@ -21075,12 +21075,12 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Jey: Steht im CRM die Bosch-Einheit "Bosch Security Systems/Building Technologies" (Grasbrunn/Straubing) oder nur andere Bosch-Gesellschaften (Robert Bosch GmbH, Rexroth, Power Tools)?</t>
+          <t>Intern klären: Steht im CRM die Bosch-Einheit "Bosch Security Systems/Building Technologies" (Grasbrunn/Straubing) oder nur andere Bosch-Gesellschaften (Robert Bosch GmbH, Rexroth, Power Tools)?</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K62" s="11" t="inlineStr"/>
@@ -21237,12 +21237,12 @@
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist MAIR Elektronik GmbH im CRM als Teil von RAWE Electronic GmbH (Zeile 1948) oder Demmel AG (Zeile 501) bereits betreut?</t>
+          <t>Intern klären: Ist MAIR Elektronik GmbH im CRM als Teil von RAWE Electronic GmbH (Zeile 1948) oder Demmel AG (Zeile 501) bereits betreut?</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K65" s="8" t="inlineStr"/>
@@ -23832,7 +23832,7 @@
       </c>
       <c r="J44" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K44" s="11" t="inlineStr"/>
@@ -27337,7 +27337,7 @@
       </c>
       <c r="I109" s="8" t="inlineStr">
         <is>
-          <t>Jey: Ist die Bürkert GmbH &amp; Co. KG im CRM (Zeile 366) Bestandskontakt der Bürkert-Gruppe, und gilt die Fäth GmbH als Schwester/Beteiligung (Rot E5 nur bei derselben Einheit; sonst Neukontakt nach Jeys Entscheidung)?</t>
+          <t>Intern klären: Ist die Bürkert GmbH &amp; Co. KG im CRM (Zeile 366) Bestandskontakt der Bürkert-Gruppe, und gilt die Fäth GmbH als Schwester/Beteiligung (Rot E5 nur bei derselben Einheit; sonst Neukontakt nach interner Entscheidung)?</t>
         </is>
       </c>
       <c r="J109" s="8" t="inlineStr">
@@ -27504,7 +27504,7 @@
       </c>
       <c r="J112" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K112" s="11" t="inlineStr"/>
@@ -27823,7 +27823,7 @@
       </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist die CRM-Einheit "VON ARDENNE GmbH" (Dresden) Gesellschafterin/Muttergesellschaft der scia Systems GmbH, und gilt der Bestandskontakt auch für scia?</t>
+          <t>Intern klären: Ist die CRM-Einheit "VON ARDENNE GmbH" (Dresden) Gesellschafterin/Muttergesellschaft der scia Systems GmbH, und gilt der Bestandskontakt auch für scia?</t>
         </is>
       </c>
       <c r="J118" s="11" t="inlineStr">
@@ -27877,12 +27877,12 @@
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Jey: Welche Gesellschaft steht hinter CRM-Zeilen "Sumitomo"/"SUMITOMO" (2273/2274)? Gehört sie zur Sumitomo-Electric-Gruppe?</t>
+          <t>Intern klären: Welche Gesellschaft steht hinter CRM-Zeilen "Sumitomo"/"SUMITOMO" (2273/2274)? Gehört sie zur Sumitomo-Electric-Gruppe?</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
       <c r="K119" s="8" t="inlineStr"/>
@@ -31992,7 +31992,7 @@
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -35107,12 +35107,12 @@
       </c>
       <c r="I135" s="8" t="inlineStr">
         <is>
-          <t>Jey: Gilt die Bosch-Gruppe im CRM als Konzernbezug für die ITK Engineering GmbH (Tochter, eigener Sitz)? (2) Hat ITK in Rülzheim eine Hardware-/Gerätefertigung (Prototypen, Kleinserie, Medizingeräte) oder reine Entwicklung (E2 …</t>
+          <t>Intern klären: Gilt die Bosch-Gruppe im CRM als Konzernbezug für die ITK Engineering GmbH (Tochter, eigener Sitz)? (2) Hat ITK in Rülzheim eine Hardware-/Gerätefertigung (Prototypen, Kleinserie, Medizingeräte) oder reine Entwicklung (E2 …</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -37447,7 +37447,7 @@
       </c>
       <c r="I180" s="11" t="inlineStr">
         <is>
-          <t>Jey: Greift E1 für die Nordson-Einheit Test &amp; Inspection (gleicher Konzern wie Dosier-Wettbewerber) oder wird sie als Kunde bewertet? (2) Falls Kunde: Wird in Feldkirchen gefertigt/montiert? Wo: Impressum nordson.com/de …</t>
+          <t>Intern klären: Greift E1 für die Nordson-Einheit Test &amp; Inspection (gleicher Konzern wie Dosier-Wettbewerber) oder wird sie als Kunde bewertet? (2) Falls Kunde: Wird in Feldkirchen gefertigt/montiert? Wo: Impressum nordson.com/de …</t>
         </is>
       </c>
       <c r="J180" s="11" t="inlineStr">
@@ -38024,7 +38024,7 @@
       </c>
       <c r="J191" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -38700,7 +38700,7 @@
       </c>
       <c r="J204" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -40255,12 +40255,12 @@
       </c>
       <c r="I234" s="11" t="inlineStr">
         <is>
-          <t>Jey: Ist CRM-Zeile 2030 "rtg electronics GmbH" dieselbe Gesellschaft wie die Tochter von SE Spezial-Electronic (Bückeburg)?</t>
+          <t>Intern klären: Ist CRM-Zeile 2030 "rtg electronics GmbH" dieselbe Gesellschaft wie die Tochter von SE Spezial-Electronic (Bückeburg)?</t>
         </is>
       </c>
       <c r="J234" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -40619,12 +40619,12 @@
       </c>
       <c r="I241" s="8" t="inlineStr">
         <is>
-          <t>Jey/Tina: Ist die CRM-Einheit "Robert Bosch GmbH" überhaupt die Einheit, aus der Immenstadt hervorging, und zählt der Altkonzern nach dem Verkauf an Sintokogio noch? Wo: Impressum und Handelsregister Sinto Advanced Ceramics …</t>
+          <t>Intern klären: Ist die CRM-Einheit "Robert Bosch GmbH" überhaupt die Einheit, aus der Immenstadt hervorging, und zählt der Altkonzern nach dem Verkauf an Sintokogio noch? Wo: Impressum und Handelsregister Sinto Advanced Ceramics …</t>
         </is>
       </c>
       <c r="J241" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -41035,12 +41035,12 @@
       </c>
       <c r="I249" s="8" t="inlineStr">
         <is>
-          <t>Jey/CRM: Ort der CRM-Einträge Phytron GmbH (Zeile 1821), FRANK Elektronik GmbH (826), EPS (715) gegen Gröbenzell, Traunstein bzw. EPS-Standort in Stemas-Gruppe abgleichen (Kundendatenbank/Registerauszug). (b) Beteiligungen ohne …</t>
+          <t>Intern klären: Ort der CRM-Einträge Phytron GmbH (Zeile 1821), FRANK Elektronik GmbH (826), EPS (715) gegen Gröbenzell, Traunstein bzw. EPS-Standort in Stemas-Gruppe abgleichen (Kundendatenbank/Registerauszug). (b) Beteiligungen ohne …</t>
         </is>
       </c>
       <c r="J249" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -42075,12 +42075,12 @@
       </c>
       <c r="I269" s="8" t="inlineStr">
         <is>
-          <t>Ist OPTEK [DE] im CRM die TT-Tochter Optek Technology oder eine andere Einheit? Wo: CRM-Datensatz (Jey/Excel), Ort der CRM-Einheit. (2) Gehört AB Elektronik GmbH Werne zu den Firmen, die auf der Messe unter "TT Electronics" …</t>
+          <t>Ist OPTEK [DE] im CRM die TT-Tochter Optek Technology oder eine andere Einheit? Wo: CRM-Datensatz (Excel), Ort der CRM-Einheit. (2) Gehört AB Elektronik GmbH Werne zu den Firmen, die auf der Messe unter "TT Electronics" …</t>
         </is>
       </c>
       <c r="J269" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -43677,12 +43677,12 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -43721,7 +43721,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -43765,7 +43765,7 @@
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
@@ -43809,7 +43809,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -43853,7 +43853,7 @@
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -43897,7 +43897,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr">
@@ -43941,7 +43941,7 @@
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
@@ -43985,7 +43985,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -44037,12 +44037,12 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -44081,7 +44081,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr">
@@ -44177,7 +44177,7 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
@@ -44221,7 +44221,7 @@
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -44265,7 +44265,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
@@ -44309,7 +44309,7 @@
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -44353,7 +44353,7 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
@@ -44405,7 +44405,7 @@
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J21" s="8" t="inlineStr">
@@ -44457,12 +44457,12 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -44509,12 +44509,12 @@
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -44561,12 +44561,12 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -44613,7 +44613,7 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
@@ -44665,7 +44665,7 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
@@ -44717,7 +44717,7 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -44761,7 +44761,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
@@ -44805,7 +44805,7 @@
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -44857,7 +44857,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
@@ -44901,7 +44901,7 @@
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J31" s="8" t="inlineStr">
@@ -44953,12 +44953,12 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -45005,7 +45005,7 @@
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J33" s="8" t="inlineStr">
@@ -45049,7 +45049,7 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J34" s="11" t="inlineStr">
@@ -45093,7 +45093,7 @@
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J35" s="8" t="inlineStr">
@@ -45137,7 +45137,7 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr">
@@ -45233,7 +45233,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
@@ -45285,7 +45285,7 @@
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
@@ -45329,7 +45329,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
@@ -45381,12 +45381,12 @@
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J41" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -45433,7 +45433,7 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J42" s="11" t="inlineStr">
@@ -45485,7 +45485,7 @@
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J43" s="8" t="inlineStr">
@@ -45537,7 +45537,7 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J44" s="11" t="inlineStr">
@@ -45589,7 +45589,7 @@
       </c>
       <c r="I45" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J45" s="8" t="inlineStr">
@@ -45641,7 +45641,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J46" s="11" t="inlineStr">
@@ -45693,7 +45693,7 @@
       </c>
       <c r="I47" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J47" s="8" t="inlineStr">
@@ -45745,7 +45745,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
@@ -45797,7 +45797,7 @@
       </c>
       <c r="I49" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J49" s="8" t="inlineStr">
@@ -45841,7 +45841,7 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
@@ -45885,7 +45885,7 @@
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
@@ -45937,7 +45937,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
@@ -45981,7 +45981,7 @@
       </c>
       <c r="I53" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
@@ -46025,7 +46025,7 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
@@ -46069,7 +46069,7 @@
       </c>
       <c r="I55" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J55" s="8" t="inlineStr">
@@ -46121,12 +46121,12 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -46165,7 +46165,7 @@
       </c>
       <c r="I57" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J57" s="8" t="inlineStr">
@@ -46209,7 +46209,7 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
@@ -46253,7 +46253,7 @@
       </c>
       <c r="I59" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J59" s="8" t="inlineStr">
@@ -46305,12 +46305,12 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -46349,7 +46349,7 @@
       </c>
       <c r="I61" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J61" s="8" t="inlineStr">
@@ -46401,7 +46401,7 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr">
@@ -46453,12 +46453,12 @@
       </c>
       <c r="I63" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J63" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -46497,7 +46497,7 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr">
@@ -46541,7 +46541,7 @@
       </c>
       <c r="I65" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J65" s="8" t="inlineStr">
@@ -46585,7 +46585,7 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
@@ -46629,7 +46629,7 @@
       </c>
       <c r="I67" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J67" s="8" t="inlineStr">
@@ -46673,7 +46673,7 @@
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr">
@@ -46717,7 +46717,7 @@
       </c>
       <c r="I69" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J69" s="8" t="inlineStr">
@@ -46761,7 +46761,7 @@
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
@@ -46813,7 +46813,7 @@
       </c>
       <c r="I71" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J71" s="8" t="inlineStr">
@@ -46865,12 +46865,12 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -46909,7 +46909,7 @@
       </c>
       <c r="I73" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J73" s="8" t="inlineStr">
@@ -46961,12 +46961,12 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J74" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47013,12 +47013,12 @@
       </c>
       <c r="I75" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J75" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47053,7 +47053,7 @@
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J76" s="11" t="inlineStr">
@@ -47097,7 +47097,7 @@
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J77" s="8" t="inlineStr">
@@ -47141,7 +47141,7 @@
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J78" s="11" t="inlineStr">
@@ -47185,7 +47185,7 @@
       </c>
       <c r="I79" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J79" s="8" t="inlineStr">
@@ -47229,7 +47229,7 @@
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr">
@@ -47281,12 +47281,12 @@
       </c>
       <c r="I81" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J81" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47333,12 +47333,12 @@
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47385,12 +47385,12 @@
       </c>
       <c r="I83" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J83" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47429,7 +47429,7 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr">
@@ -47481,12 +47481,12 @@
       </c>
       <c r="I85" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J85" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47533,7 +47533,7 @@
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr">
@@ -47585,12 +47585,12 @@
       </c>
       <c r="I87" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J87" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47629,7 +47629,7 @@
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr">
@@ -47673,7 +47673,7 @@
       </c>
       <c r="I89" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J89" s="8" t="inlineStr">
@@ -47717,7 +47717,7 @@
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr">
@@ -47769,12 +47769,12 @@
       </c>
       <c r="I91" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J91" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -47813,7 +47813,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J92" s="11" t="inlineStr">
@@ -47865,7 +47865,7 @@
       </c>
       <c r="I93" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J93" s="8" t="inlineStr">
@@ -47909,7 +47909,7 @@
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J94" s="11" t="inlineStr">
@@ -47953,7 +47953,7 @@
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J95" s="8" t="inlineStr">
@@ -47997,7 +47997,7 @@
       </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J96" s="11" t="inlineStr">
@@ -48041,7 +48041,7 @@
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J97" s="8" t="inlineStr">
@@ -48089,12 +48089,12 @@
       </c>
       <c r="I98" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J98" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -48141,12 +48141,12 @@
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J99" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -48185,7 +48185,7 @@
       </c>
       <c r="I100" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J100" s="11" t="inlineStr">
@@ -48229,7 +48229,7 @@
       </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
@@ -48273,7 +48273,7 @@
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J102" s="11" t="inlineStr">
@@ -48325,12 +48325,12 @@
       </c>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J103" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -48369,7 +48369,7 @@
       </c>
       <c r="I104" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J104" s="11" t="inlineStr">
@@ -48421,7 +48421,7 @@
       </c>
       <c r="I105" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J105" s="8" t="inlineStr">
@@ -48473,12 +48473,12 @@
       </c>
       <c r="I106" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J106" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -48517,7 +48517,7 @@
       </c>
       <c r="I107" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J107" s="8" t="inlineStr">
@@ -48561,7 +48561,7 @@
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J108" s="11" t="inlineStr">
@@ -48605,7 +48605,7 @@
       </c>
       <c r="I109" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J109" s="8" t="inlineStr">
@@ -48649,7 +48649,7 @@
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr">
@@ -48693,7 +48693,7 @@
       </c>
       <c r="I111" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J111" s="8" t="inlineStr">
@@ -48737,7 +48737,7 @@
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J112" s="11" t="inlineStr">
@@ -48781,7 +48781,7 @@
       </c>
       <c r="I113" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J113" s="8" t="inlineStr">
@@ -48825,7 +48825,7 @@
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J114" s="11" t="inlineStr">
@@ -48869,7 +48869,7 @@
       </c>
       <c r="I115" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J115" s="8" t="inlineStr">
@@ -48913,7 +48913,7 @@
       </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J116" s="11" t="inlineStr">
@@ -48965,12 +48965,12 @@
       </c>
       <c r="I117" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J117" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49009,7 +49009,7 @@
       </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J118" s="11" t="inlineStr">
@@ -49053,7 +49053,7 @@
       </c>
       <c r="I119" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J119" s="8" t="inlineStr">
@@ -49105,12 +49105,12 @@
       </c>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J120" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49157,7 +49157,7 @@
       </c>
       <c r="I121" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J121" s="8" t="inlineStr">
@@ -49209,7 +49209,7 @@
       </c>
       <c r="I122" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J122" s="11" t="inlineStr">
@@ -49261,7 +49261,7 @@
       </c>
       <c r="I123" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J123" s="8" t="inlineStr">
@@ -49305,7 +49305,7 @@
       </c>
       <c r="I124" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J124" s="11" t="inlineStr">
@@ -49349,7 +49349,7 @@
       </c>
       <c r="I125" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J125" s="8" t="inlineStr">
@@ -49401,12 +49401,12 @@
       </c>
       <c r="I126" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J126" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49445,7 +49445,7 @@
       </c>
       <c r="I127" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J127" s="8" t="inlineStr">
@@ -49497,12 +49497,12 @@
       </c>
       <c r="I128" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J128" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49549,12 +49549,12 @@
       </c>
       <c r="I129" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J129" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49601,12 +49601,12 @@
       </c>
       <c r="I130" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J130" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49653,12 +49653,12 @@
       </c>
       <c r="I131" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J131" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -49697,7 +49697,7 @@
       </c>
       <c r="I132" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J132" s="11" t="inlineStr">
@@ -49741,7 +49741,7 @@
       </c>
       <c r="I133" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J133" s="8" t="inlineStr">
@@ -49793,7 +49793,7 @@
       </c>
       <c r="I134" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J134" s="11" t="inlineStr">
@@ -49837,7 +49837,7 @@
       </c>
       <c r="I135" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J135" s="8" t="inlineStr">
@@ -49889,7 +49889,7 @@
       </c>
       <c r="I136" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J136" s="11" t="inlineStr">
@@ -49933,7 +49933,7 @@
       </c>
       <c r="I137" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J137" s="8" t="inlineStr">
@@ -49977,7 +49977,7 @@
       </c>
       <c r="I138" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J138" s="11" t="inlineStr">
@@ -50029,7 +50029,7 @@
       </c>
       <c r="I139" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J139" s="8" t="inlineStr">
@@ -50081,7 +50081,7 @@
       </c>
       <c r="I140" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J140" s="11" t="inlineStr">
@@ -50125,7 +50125,7 @@
       </c>
       <c r="I141" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J141" s="8" t="inlineStr">
@@ -50169,7 +50169,7 @@
       </c>
       <c r="I142" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J142" s="11" t="inlineStr">
@@ -50221,12 +50221,12 @@
       </c>
       <c r="I143" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J143" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -50265,7 +50265,7 @@
       </c>
       <c r="I144" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J144" s="11" t="inlineStr">
@@ -50317,7 +50317,7 @@
       </c>
       <c r="I145" s="8" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J145" s="8" t="inlineStr">
@@ -50369,7 +50369,7 @@
       </c>
       <c r="I146" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J146" s="11" t="inlineStr">
@@ -50413,7 +50413,7 @@
       </c>
       <c r="I147" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J147" s="8" t="inlineStr">
@@ -50465,7 +50465,7 @@
       </c>
       <c r="I148" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J148" s="11" t="inlineStr">
@@ -50517,12 +50517,12 @@
       </c>
       <c r="I149" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J149" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -50561,7 +50561,7 @@
       </c>
       <c r="I150" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J150" s="11" t="inlineStr">
@@ -50605,7 +50605,7 @@
       </c>
       <c r="I151" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J151" s="8" t="inlineStr">
@@ -50649,7 +50649,7 @@
       </c>
       <c r="I152" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J152" s="11" t="inlineStr">
@@ -50693,7 +50693,7 @@
       </c>
       <c r="I153" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J153" s="8" t="inlineStr">
@@ -50745,7 +50745,7 @@
       </c>
       <c r="I154" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J154" s="11" t="inlineStr">
@@ -50789,7 +50789,7 @@
       </c>
       <c r="I155" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J155" s="8" t="inlineStr">
@@ -50841,7 +50841,7 @@
       </c>
       <c r="I156" s="11" t="inlineStr">
         <is>
-          <t>Verband / Prüfdienstleister / Forschung – laut Jey raus</t>
+          <t>Verband / Prüfdienstleister / Forschung</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr">
@@ -50893,12 +50893,12 @@
       </c>
       <c r="I157" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J157" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -50937,7 +50937,7 @@
       </c>
       <c r="I158" s="11" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J158" s="11" t="inlineStr">
@@ -50989,12 +50989,12 @@
       </c>
       <c r="I159" s="8" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J159" s="8" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -51041,12 +51041,12 @@
       </c>
       <c r="I160" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J160" s="11" t="inlineStr">
         <is>
-          <t>Konzern/ähnlicher Name im CRM – Jey klären</t>
+          <t>Konzern-/ähnlicher Name im CRM – vor Kontakt intern klären</t>
         </is>
       </c>
     </row>
@@ -51085,7 +51085,7 @@
       </c>
       <c r="I161" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J161" s="8" t="inlineStr">
@@ -51137,7 +51137,7 @@
       </c>
       <c r="I162" s="11" t="inlineStr">
         <is>
-          <t>Im CRM (gleicher oder sehr ähnlicher Name) – laut Jey raus</t>
+          <t>Im CRM (gleicher oder sehr ähnlicher Name)</t>
         </is>
       </c>
       <c r="J162" s="11" t="inlineStr">
@@ -51181,7 +51181,7 @@
       </c>
       <c r="I163" s="8" t="inlineStr">
         <is>
-          <t>Bestandskunde laut CRM-Abgleich (Namensabgleich, nicht durch Tom/Tina geprüft) – Zuständigen im Haus fragen</t>
+          <t>Bestandskunde laut CRM-Namensabgleich – nicht ansprechen, Zuständigen im Haus fragen</t>
         </is>
       </c>
       <c r="J163" s="8" t="inlineStr">
@@ -51257,7 +51257,7 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Zuerst Identität oder CRM-Bezug klären (z. B. Konzern im CRM, Sitz unklar). Nicht ohne Rückmeldung von Jey kontaktieren.</t>
+          <t>Zuerst Identität oder CRM-Bezug klären (z. B. Konzern im CRM, Sitz unklar). Nicht ohne interne Rückmeldung kontaktieren.</t>
         </is>
       </c>
     </row>
@@ -51293,7 +51293,7 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>Alles, was laut Jey rausfällt: (1) Firmen im CRM mit gleichem oder sehr ähnlichem Namen (88 Namensabgleich-Treffer plus Tom/Tina-Treffer inkl. Konzernname), (2) Verbände, Prüfdienstleister, Forschungsorganisationen, (3) Anlagenbauer ohne Verguss-/Demak-Anlage. Grund steht in Spalte "Vor dem Kontakt klären".</t>
+          <t>Alles, was nicht angesprochen wird: (1) Firmen im CRM mit gleichem oder sehr ähnlichem Namen (88 Namensabgleich-Treffer plus Treffer aus der Recherche inkl. Konzernname), (2) Verbände, Prüfdienstleister, Forschungsorganisationen, (3) Anlagenbauer ohne Verguss-/Demak-Anlage. Grund steht in Spalte "Vor dem Kontakt klären".</t>
         </is>
       </c>
     </row>
@@ -51341,7 +51341,7 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Nicht geprüft. Eigenfertigung und Wettbewerbereinsatz im Gespräch erfragen.</t>
+          <t>Patente nur bei den 46 Browser-geprüften Firmen (Google Patents, Espacenet) gesucht. Eigenfertigung und Wettbewerbereinsatz im Gespräch erfragen.</t>
         </is>
       </c>
     </row>
@@ -51353,7 +51353,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Tom/Tina. Zuständig: Stefan = Baden-Württemberg, Dietmar = Bayern, Manuel = Rest DE / NL. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
+          <t>Pro Vertriebsgebiet ein Blatt (Baden-Württemberg, Bayern, Rest DE / NL, ggf. Österreich/außerhalb; nur Prio A/B/C). Gebiet nach Fertigungs- bzw. Firmensitz laut Recherche. Zuständig: Stefan = Baden-Württemberg, Dietmar = Bayern, Manuel = Rest DE / NL. Das Blatt "Zielfirmen" enthält alle zusammen.</t>
         </is>
       </c>
     </row>

</xml_diff>